<commit_message>
Fix broken string references
The string table had duplicate entries for the same tring ID. This impacts some Phoenix Armoury and the Garahel item sets. New string references have been generated and the items updated to use them.

closes #400
</commit_message>
<xml_diff>
--- a/source/tlk/strings.xlsx
+++ b/source/tlk/strings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\DAO\archid\source\tlk\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A208C17-F6EE-4F93-846F-53AEDFC424DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD74EB2B-E1F4-414F-95E3-4646B7E60C0E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2865" yWindow="615" windowWidth="23640" windowHeight="16110" xr2:uid="{A42EE72D-E1C4-43B6-AEA5-0014ED5180B1}"/>
+    <workbookView xWindow="29610" yWindow="600" windowWidth="23640" windowHeight="16110" xr2:uid="{A42EE72D-E1C4-43B6-AEA5-0014ED5180B1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -5048,7 +5048,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -5069,6 +5069,8 @@
     </xf>
     <xf numFmtId="49" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -12421,161 +12423,161 @@
     </row>
     <row r="879" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A879" s="5">
-        <v>6610845</v>
-      </c>
-      <c r="B879" s="3" t="s">
+        <v>6610877</v>
+      </c>
+      <c r="B879" s="12" t="s">
         <v>1478</v>
       </c>
     </row>
     <row r="880" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A880" s="5">
-        <v>6610846</v>
-      </c>
-      <c r="B880" s="3" t="s">
+        <v>6610878</v>
+      </c>
+      <c r="B880" s="12" t="s">
         <v>1498</v>
       </c>
     </row>
     <row r="881" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A881" s="5">
-        <v>6610847</v>
-      </c>
-      <c r="B881" s="3" t="s">
+        <v>6610879</v>
+      </c>
+      <c r="B881" s="12" t="s">
         <v>1479</v>
       </c>
     </row>
     <row r="882" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A882" s="5">
-        <v>6610848</v>
-      </c>
-      <c r="B882" s="3" t="s">
+        <v>6610880</v>
+      </c>
+      <c r="B882" s="12" t="s">
         <v>1501</v>
       </c>
     </row>
     <row r="883" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A883" s="5">
-        <v>6610849</v>
-      </c>
-      <c r="B883" s="3" t="s">
+        <v>6610881</v>
+      </c>
+      <c r="B883" s="12" t="s">
         <v>1480</v>
       </c>
     </row>
     <row r="884" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A884" s="5">
-        <v>6610850</v>
-      </c>
-      <c r="B884" s="3" t="s">
+        <v>6610882</v>
+      </c>
+      <c r="B884" s="12" t="s">
         <v>1502</v>
       </c>
     </row>
     <row r="885" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A885" s="5">
-        <v>6610851</v>
-      </c>
-      <c r="B885" s="3" t="s">
+        <v>6610883</v>
+      </c>
+      <c r="B885" s="12" t="s">
         <v>1481</v>
       </c>
     </row>
     <row r="886" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A886" s="5">
-        <v>6610852</v>
-      </c>
-      <c r="B886" s="3" t="s">
+        <v>6610884</v>
+      </c>
+      <c r="B886" s="12" t="s">
         <v>1496</v>
       </c>
     </row>
     <row r="887" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A887" s="5">
-        <v>6610853</v>
-      </c>
-      <c r="B887" s="3" t="s">
+        <v>6610885</v>
+      </c>
+      <c r="B887" s="12" t="s">
         <v>1482</v>
       </c>
     </row>
     <row r="888" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A888" s="5">
-        <v>6610854</v>
-      </c>
-      <c r="B888" s="3" t="s">
+        <v>6610886</v>
+      </c>
+      <c r="B888" s="12" t="s">
         <v>1499</v>
       </c>
     </row>
     <row r="889" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A889" s="4">
-        <v>6610855</v>
-      </c>
-      <c r="B889" s="11" t="s">
+        <v>6610887</v>
+      </c>
+      <c r="B889" s="13" t="s">
         <v>1504</v>
       </c>
     </row>
     <row r="890" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A890" s="4">
-        <v>6610856</v>
-      </c>
-      <c r="B890" s="11" t="s">
+        <v>6610888</v>
+      </c>
+      <c r="B890" s="13" t="s">
         <v>1505</v>
       </c>
     </row>
     <row r="891" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A891" s="4">
-        <v>6610857</v>
-      </c>
-      <c r="B891" s="11" t="s">
+        <v>6610889</v>
+      </c>
+      <c r="B891" s="13" t="s">
         <v>1506</v>
       </c>
     </row>
     <row r="892" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A892" s="4">
-        <v>6610858</v>
-      </c>
-      <c r="B892" s="11" t="s">
+        <v>6610890</v>
+      </c>
+      <c r="B892" s="13" t="s">
         <v>1505</v>
       </c>
     </row>
     <row r="893" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A893" s="4">
-        <v>6610859</v>
-      </c>
-      <c r="B893" s="11" t="s">
+        <v>6610891</v>
+      </c>
+      <c r="B893" s="13" t="s">
         <v>1507</v>
       </c>
     </row>
     <row r="894" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A894" s="4">
-        <v>6610860</v>
-      </c>
-      <c r="B894" s="11" t="s">
+        <v>6610892</v>
+      </c>
+      <c r="B894" s="13" t="s">
         <v>1505</v>
       </c>
     </row>
     <row r="895" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A895" s="4">
-        <v>6610861</v>
-      </c>
-      <c r="B895" s="11" t="s">
+        <v>6610893</v>
+      </c>
+      <c r="B895" s="13" t="s">
         <v>1508</v>
       </c>
     </row>
     <row r="896" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A896" s="4">
-        <v>6610862</v>
-      </c>
-      <c r="B896" s="11" t="s">
+        <v>6610894</v>
+      </c>
+      <c r="B896" s="13" t="s">
         <v>1509</v>
       </c>
     </row>
     <row r="897" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A897" s="4">
-        <v>6610863</v>
-      </c>
-      <c r="B897" s="11" t="s">
+        <v>6610895</v>
+      </c>
+      <c r="B897" s="13" t="s">
         <v>1510</v>
       </c>
     </row>
     <row r="898" spans="1:2" s="11" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A898" s="4">
-        <v>6610864</v>
-      </c>
-      <c r="B898" s="11" t="s">
+        <v>6610896</v>
+      </c>
+      <c r="B898" s="13" t="s">
         <v>1509</v>
       </c>
     </row>

</xml_diff>